<commit_message>
Fix all 18 SEO audit issues: security headers, canonicals, meta descriptions, alt text, URL params, image sizes, noindex pages
</commit_message>
<xml_diff>
--- a/SEO Files/issues_overview_report.xlsx
+++ b/SEO Files/issues_overview_report.xlsx
@@ -118,10 +118,10 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>21.0</v>
+        <v>10.0</v>
       </c>
       <c r="E2" t="n">
-        <v>91.3</v>
+        <v>43.48</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -186,10 +186,10 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>21.0</v>
+        <v>10.0</v>
       </c>
       <c r="E4" t="n">
-        <v>91.3</v>
+        <v>43.48</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -220,10 +220,10 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>21.0</v>
+        <v>2.0</v>
       </c>
       <c r="E5" t="n">
-        <v>91.3</v>
+        <v>8.7</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -356,10 +356,10 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>21.0</v>
+        <v>2.0</v>
       </c>
       <c r="E9" t="n">
-        <v>91.3</v>
+        <v>8.7</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
@@ -662,10 +662,10 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>21.0</v>
+        <v>2.0</v>
       </c>
       <c r="E18" t="n">
-        <v>91.3</v>
+        <v>8.7</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>

</xml_diff>